<commit_message>
add: driver printer epson
</commit_message>
<xml_diff>
--- a/FILE EXCEL DISINI/PRAGAAN 16-04-2026.xlsx
+++ b/FILE EXCEL DISINI/PRAGAAN 16-04-2026.xlsx
@@ -2842,108 +2842,113 @@
       <c r="AD21" t="inlineStr"/>
     </row>
     <row r="22" ht="16.5" customHeight="1" s="45">
-      <c r="A22" s="11" t="n">
+      <c r="A22" s="46" t="n">
         <v>19</v>
       </c>
-      <c r="B22" s="20" t="inlineStr">
+      <c r="B22" s="49" t="inlineStr">
         <is>
           <t>DIKAN</t>
         </is>
       </c>
-      <c r="C22" s="34" t="inlineStr">
+      <c r="C22" s="48" t="inlineStr">
         <is>
           <t>HT</t>
         </is>
       </c>
-      <c r="D22" s="20" t="n">
+      <c r="D22" s="49" t="n">
         <v>779181388</v>
       </c>
-      <c r="E22" s="40" t="inlineStr">
+      <c r="E22" s="50" t="inlineStr">
         <is>
           <t>3529116004710001</t>
         </is>
       </c>
-      <c r="F22" s="37" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="15" t="n"/>
-      <c r="I22" s="16" t="n">
+      <c r="F22" s="51" t="n"/>
+      <c r="G22" s="52" t="n"/>
+      <c r="H22" s="53" t="n"/>
+      <c r="I22" s="54" t="n">
         <v>135</v>
       </c>
-      <c r="J22" s="16" t="n">
+      <c r="J22" s="54" t="n">
         <v>250</v>
       </c>
-      <c r="K22" s="16" t="n">
+      <c r="K22" s="54" t="n">
         <v>35</v>
       </c>
-      <c r="L22" s="17" t="n">
+      <c r="L22" s="55" t="n">
         <v>0.7</v>
       </c>
-      <c r="M22" s="16" t="n">
+      <c r="M22" s="54" t="n">
         <v>74</v>
       </c>
-      <c r="N22" s="16" t="n">
+      <c r="N22" s="54" t="n">
         <v>11</v>
       </c>
-      <c r="O22" s="18" t="n"/>
-      <c r="P22" s="19" t="n">
+      <c r="O22" s="56" t="n"/>
+      <c r="P22" s="57" t="n">
         <v>71.3</v>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="Q22" s="58" t="inlineStr">
         <is>
           <t>16-04-2026</t>
         </is>
       </c>
-      <c r="R22" s="42" t="inlineStr">
-        <is>
-          <t>SUKSES</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr">
+      <c r="R22" s="59" t="inlineStr">
+        <is>
+          <t>SUKSES</t>
+        </is>
+      </c>
+      <c r="S22" s="58" t="inlineStr">
+        <is>
+          <t>SUKSES</t>
+        </is>
+      </c>
+      <c r="T22" s="58" t="inlineStr">
         <is>
           <t>36.5</t>
         </is>
       </c>
-      <c r="U22" t="inlineStr">
+      <c r="U22" s="58" t="inlineStr">
         <is>
           <t>158</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="V22" s="58" t="inlineStr">
         <is>
           <t>54</t>
         </is>
       </c>
-      <c r="W22" t="inlineStr">
+      <c r="W22" s="58" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="X22" t="inlineStr">
+      <c r="X22" s="58" t="inlineStr">
         <is>
           <t>21.63</t>
         </is>
       </c>
-      <c r="Y22" t="inlineStr">
+      <c r="Y22" s="58" t="inlineStr">
         <is>
           <t>150</t>
         </is>
       </c>
-      <c r="Z22" t="inlineStr">
+      <c r="Z22" s="58" t="inlineStr">
         <is>
           <t>90</t>
         </is>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AA22" s="58" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="AB22" t="inlineStr">
+      <c r="AB22" s="58" t="inlineStr">
         <is>
           <t>80</t>
         </is>
       </c>
-      <c r="AC22" t="inlineStr">
+      <c r="AC22" s="58" t="inlineStr">
         <is>
           <t>FINISH</t>
         </is>
@@ -2951,62 +2956,118 @@
       <c r="AD22" t="inlineStr"/>
     </row>
     <row r="23" ht="16.5" customHeight="1" s="45">
-      <c r="A23" s="11" t="n">
+      <c r="A23" s="46" t="n">
         <v>20</v>
       </c>
-      <c r="B23" s="20" t="inlineStr">
+      <c r="B23" s="49" t="inlineStr">
         <is>
           <t>DIYANI</t>
         </is>
       </c>
-      <c r="C23" s="34" t="inlineStr">
+      <c r="C23" s="48" t="inlineStr">
         <is>
           <t>HT</t>
         </is>
       </c>
-      <c r="D23" s="20" t="n">
+      <c r="D23" s="49" t="n">
         <v>778658848</v>
       </c>
-      <c r="E23" s="40" t="inlineStr">
+      <c r="E23" s="50" t="inlineStr">
         <is>
           <t>3529114602610003</t>
         </is>
       </c>
-      <c r="F23" s="37" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="15" t="n"/>
-      <c r="I23" s="16" t="n">
+      <c r="F23" s="51" t="n"/>
+      <c r="G23" s="52" t="n"/>
+      <c r="H23" s="53" t="n"/>
+      <c r="I23" s="54" t="n">
         <v>282</v>
       </c>
-      <c r="J23" s="16" t="n">
+      <c r="J23" s="54" t="n">
         <v>302</v>
       </c>
-      <c r="K23" s="16" t="n">
+      <c r="K23" s="54" t="n">
         <v>29</v>
       </c>
-      <c r="L23" s="17" t="n">
+      <c r="L23" s="55" t="n">
         <v>0.7</v>
       </c>
-      <c r="M23" s="16" t="n">
+      <c r="M23" s="54" t="n">
         <v>88</v>
       </c>
-      <c r="N23" s="16" t="n">
+      <c r="N23" s="54" t="n">
         <v>134</v>
       </c>
-      <c r="O23" s="18" t="n"/>
-      <c r="P23" s="19" t="n">
+      <c r="O23" s="56" t="n"/>
+      <c r="P23" s="57" t="n">
         <v>26.7</v>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="Q23" s="58" t="inlineStr">
         <is>
           <t>16-04-2026</t>
         </is>
       </c>
-      <c r="R23" s="42" t="inlineStr">
-        <is>
-          <t>SUKSES</t>
-        </is>
-      </c>
+      <c r="R23" s="59" t="inlineStr">
+        <is>
+          <t>SUKSES</t>
+        </is>
+      </c>
+      <c r="S23" s="58" t="inlineStr">
+        <is>
+          <t>SUKSES</t>
+        </is>
+      </c>
+      <c r="T23" s="58" t="inlineStr">
+        <is>
+          <t>36.2</t>
+        </is>
+      </c>
+      <c r="U23" s="58" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="V23" s="58" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="W23" s="58" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="X23" s="58" t="inlineStr">
+        <is>
+          <t>22.22</t>
+        </is>
+      </c>
+      <c r="Y23" s="58" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="Z23" s="58" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="AA23" s="58" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="AB23" s="58" t="inlineStr">
+        <is>
+          <t>80</t>
+        </is>
+      </c>
+      <c r="AC23" s="58" t="inlineStr">
+        <is>
+          <t>FINISH</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr"/>
     </row>
     <row r="24" ht="16.5" customHeight="1" s="45">
       <c r="A24" s="11" t="n">

</xml_diff>